<commit_message>
Update MLB weather 2026-07-22 07:56 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_07_23.xlsx
+++ b/mlb_weather_professional_v5_2026_07_23.xlsx
@@ -356,7 +356,7 @@
     <t>🟨 Neutral</t>
   </si>
   <si>
-    <t>WORSENING</t>
+    <t>STEADY</t>
   </si>
   <si>
     <t>WORSENING RAPIDLY</t>
@@ -371,16 +371,16 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-22 07:56:39 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-22 07:56:40 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-22 07:56:41 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-22 07:56:42 PM PDT</t>
+    <t>2026-07-22 07:56:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-22 07:56:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-22 07:56:55 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-22 07:56:56 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -725,16 +725,16 @@
     <t>09:40 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-23 02:56:39 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-23 02:56:40 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-23 02:56:41 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-23 02:56:42 UTC</t>
+    <t>2026-07-23 02:56:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-23 02:56:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-23 02:56:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-23 02:56:56 UTC</t>
   </si>
   <si>
     <t>2026-07-23T00:12:17+00:00</t>
@@ -1600,7 +1600,7 @@
         <v>111</v>
       </c>
       <c r="AR2">
-        <v>-1.5</v>
+        <v>-1.1</v>
       </c>
       <c r="AS2">
         <v>0</v>
@@ -1624,7 +1624,7 @@
         <v>116</v>
       </c>
       <c r="AZ2">
-        <v>164.4</v>
+        <v>164.6</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -1758,7 +1758,7 @@
         <v>112</v>
       </c>
       <c r="AR3">
-        <v>-7.8</v>
+        <v>-7.9</v>
       </c>
       <c r="AS3">
         <v>0</v>
@@ -1782,7 +1782,7 @@
         <v>117</v>
       </c>
       <c r="AZ3">
-        <v>429.3</v>
+        <v>429.6</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -1916,7 +1916,7 @@
         <v>113</v>
       </c>
       <c r="AR4">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="AS4">
         <v>0</v>
@@ -1937,7 +1937,7 @@
         <v>1.6</v>
       </c>
       <c r="AY4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AZ4">
         <v>0</v>
@@ -2074,7 +2074,7 @@
         <v>112</v>
       </c>
       <c r="AR5">
-        <v>-6.3</v>
+        <v>-7.2</v>
       </c>
       <c r="AS5">
         <v>0</v>
@@ -2095,10 +2095,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="AY5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AZ5">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2232,7 +2232,7 @@
         <v>112</v>
       </c>
       <c r="AR6">
-        <v>-7.8</v>
+        <v>-8</v>
       </c>
       <c r="AS6">
         <v>0</v>
@@ -2256,7 +2256,7 @@
         <v>119</v>
       </c>
       <c r="AZ6">
-        <v>343.2</v>
+        <v>343.4</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2726,7 +2726,7 @@
         <v>238</v>
       </c>
       <c r="J2">
-        <v>164.4</v>
+        <v>164.6</v>
       </c>
       <c r="K2">
         <v>13.3</v>
@@ -3040,7 +3040,7 @@
         <v>238</v>
       </c>
       <c r="J3">
-        <v>164.4</v>
+        <v>164.6</v>
       </c>
       <c r="K3">
         <v>14.3</v>
@@ -3354,7 +3354,7 @@
         <v>238</v>
       </c>
       <c r="J4">
-        <v>164.4</v>
+        <v>164.6</v>
       </c>
       <c r="K4">
         <v>15.3</v>
@@ -3668,7 +3668,7 @@
         <v>238</v>
       </c>
       <c r="J5">
-        <v>164.4</v>
+        <v>164.6</v>
       </c>
       <c r="K5">
         <v>16.3</v>
@@ -3982,7 +3982,7 @@
         <v>239</v>
       </c>
       <c r="J6">
-        <v>429.3</v>
+        <v>429.6</v>
       </c>
       <c r="K6">
         <v>14.2</v>
@@ -4296,7 +4296,7 @@
         <v>239</v>
       </c>
       <c r="J7">
-        <v>429.3</v>
+        <v>429.6</v>
       </c>
       <c r="K7">
         <v>15.2</v>
@@ -4610,7 +4610,7 @@
         <v>239</v>
       </c>
       <c r="J8">
-        <v>429.3</v>
+        <v>429.6</v>
       </c>
       <c r="K8">
         <v>16.2</v>
@@ -4924,7 +4924,7 @@
         <v>239</v>
       </c>
       <c r="J9">
-        <v>429.3</v>
+        <v>429.6</v>
       </c>
       <c r="K9">
         <v>17.2</v>
@@ -5229,10 +5229,10 @@
         <v>76</v>
       </c>
       <c r="G10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -5537,10 +5537,10 @@
         <v>225</v>
       </c>
       <c r="G11" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H11" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -5845,10 +5845,10 @@
         <v>226</v>
       </c>
       <c r="G12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -6153,10 +6153,10 @@
         <v>227</v>
       </c>
       <c r="G13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -6461,16 +6461,16 @@
         <v>77</v>
       </c>
       <c r="G14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I14" t="s">
         <v>240</v>
       </c>
       <c r="J14">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="K14">
         <v>18.3</v>
@@ -6775,16 +6775,16 @@
         <v>228</v>
       </c>
       <c r="G15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I15" t="s">
         <v>240</v>
       </c>
       <c r="J15">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="K15">
         <v>19.3</v>
@@ -7089,16 +7089,16 @@
         <v>229</v>
       </c>
       <c r="G16" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I16" t="s">
         <v>240</v>
       </c>
       <c r="J16">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="K16">
         <v>20.3</v>
@@ -7403,16 +7403,16 @@
         <v>230</v>
       </c>
       <c r="G17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I17" t="s">
         <v>240</v>
       </c>
       <c r="J17">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="K17">
         <v>21.3</v>
@@ -7726,7 +7726,7 @@
         <v>241</v>
       </c>
       <c r="J18">
-        <v>343.2</v>
+        <v>343.4</v>
       </c>
       <c r="K18">
         <v>19.7</v>
@@ -8040,7 +8040,7 @@
         <v>241</v>
       </c>
       <c r="J19">
-        <v>343.2</v>
+        <v>343.4</v>
       </c>
       <c r="K19">
         <v>20.7</v>
@@ -8354,7 +8354,7 @@
         <v>241</v>
       </c>
       <c r="J20">
-        <v>343.2</v>
+        <v>343.4</v>
       </c>
       <c r="K20">
         <v>21.7</v>
@@ -8668,7 +8668,7 @@
         <v>241</v>
       </c>
       <c r="J21">
-        <v>343.2</v>
+        <v>343.4</v>
       </c>
       <c r="K21">
         <v>22.7</v>

</xml_diff>